<commit_message>
Implement deck archetype and QA pipeline
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madis\Documents\pokemon_scraper\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C96AD8B-47ED-4243-BBBD-2D885C9E5590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBBD407-B975-4D99-BB92-DD1840BF4EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tournaments" sheetId="1" r:id="rId1"/>
     <sheet name="sets" sheetId="4" r:id="rId2"/>
+    <sheet name="archetypes" sheetId="5" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">archetypes!$A$1:$F$63</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -26,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="200">
   <si>
     <t>tournament_id</t>
   </si>
@@ -281,6 +285,351 @@
   </si>
   <si>
     <t>NA01wMo4vxttnwEyqclr</t>
+  </si>
+  <si>
+    <t>overall_archetype</t>
+  </si>
+  <si>
+    <t>card_name</t>
+  </si>
+  <si>
+    <t>Dragapult</t>
+  </si>
+  <si>
+    <t>Dragapult ex</t>
+  </si>
+  <si>
+    <t>Blaziken ex</t>
+  </si>
+  <si>
+    <t>Dusknoir</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>variant</t>
+  </si>
+  <si>
+    <t>operator</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>&gt;=</t>
+  </si>
+  <si>
+    <t>Blaziken</t>
+  </si>
+  <si>
+    <t>Dudunsparce</t>
+  </si>
+  <si>
+    <t>N'z Zoroark</t>
+  </si>
+  <si>
+    <t>Straight</t>
+  </si>
+  <si>
+    <t>N's Zoroark ex</t>
+  </si>
+  <si>
+    <t>Crustle</t>
+  </si>
+  <si>
+    <t>Slowking</t>
+  </si>
+  <si>
+    <t>Hydrapple</t>
+  </si>
+  <si>
+    <t>Alakazam</t>
+  </si>
+  <si>
+    <t>Raging Bolt</t>
+  </si>
+  <si>
+    <t>Ogerpon Box</t>
+  </si>
+  <si>
+    <t>Hydrapple ex</t>
+  </si>
+  <si>
+    <t>Raging Bolt ex</t>
+  </si>
+  <si>
+    <t>Teal Mask Ogerpon ex</t>
+  </si>
+  <si>
+    <t>Wellspring Mask Ogerpon ex</t>
+  </si>
+  <si>
+    <t>Area Zero Underdepths</t>
+  </si>
+  <si>
+    <t>Lillie's Clefairy</t>
+  </si>
+  <si>
+    <t>Lillie's Clefairy ex</t>
+  </si>
+  <si>
+    <t>Rocket's Honchkrow</t>
+  </si>
+  <si>
+    <t>Team Rocket's Honchkrow</t>
+  </si>
+  <si>
+    <t>Festival Lead</t>
+  </si>
+  <si>
+    <t>Thwackey</t>
+  </si>
+  <si>
+    <t>Mega Lucario</t>
+  </si>
+  <si>
+    <t>Mega Lucario ex</t>
+  </si>
+  <si>
+    <t>Hop's Trevenant</t>
+  </si>
+  <si>
+    <t>Beedrill</t>
+  </si>
+  <si>
+    <t>Beedrill ex</t>
+  </si>
+  <si>
+    <t>Ethan's Typhlosion</t>
+  </si>
+  <si>
+    <t>Cynthia's Garchomp</t>
+  </si>
+  <si>
+    <t>Cynthia's Garchomp ex</t>
+  </si>
+  <si>
+    <t>Metagross</t>
+  </si>
+  <si>
+    <t>Mega Lopunny</t>
+  </si>
+  <si>
+    <t>Mega Lopunny ex</t>
+  </si>
+  <si>
+    <t>Wally's Compassion</t>
+  </si>
+  <si>
+    <t>Marnie's Grimmsnarl</t>
+  </si>
+  <si>
+    <t>Marnie's Grimmsnarl ex</t>
+  </si>
+  <si>
+    <t>Frosslass</t>
+  </si>
+  <si>
+    <t>Mega Starmie ex</t>
+  </si>
+  <si>
+    <t>Mega Frosslass ex</t>
+  </si>
+  <si>
+    <t>Mega Greninja</t>
+  </si>
+  <si>
+    <t>Mega Greninja ex</t>
+  </si>
+  <si>
+    <t>Ogerpon Meganium</t>
+  </si>
+  <si>
+    <t>Arboliva</t>
+  </si>
+  <si>
+    <t>Meganium</t>
+  </si>
+  <si>
+    <t>Arboliva ex</t>
+  </si>
+  <si>
+    <t>Sylveon</t>
+  </si>
+  <si>
+    <t>Archaludon</t>
+  </si>
+  <si>
+    <t>Zoroark</t>
+  </si>
+  <si>
+    <t>Archaludon ex</t>
+  </si>
+  <si>
+    <t>Ceruledge</t>
+  </si>
+  <si>
+    <t>Ceruledge ex</t>
+  </si>
+  <si>
+    <t>Greninja ex</t>
+  </si>
+  <si>
+    <t>Greninja</t>
+  </si>
+  <si>
+    <t>Mega Diancie</t>
+  </si>
+  <si>
+    <t>Mega Diancie ex</t>
+  </si>
+  <si>
+    <t>Tera Box</t>
+  </si>
+  <si>
+    <t>Noctowl</t>
+  </si>
+  <si>
+    <t>Steven's Metagross</t>
+  </si>
+  <si>
+    <t>Steven's Metagross ex</t>
+  </si>
+  <si>
+    <t>Mega Absol Box</t>
+  </si>
+  <si>
+    <t>Mega Absol ex</t>
+  </si>
+  <si>
+    <t>Toxtricity</t>
+  </si>
+  <si>
+    <t>Tank Kangaskhan</t>
+  </si>
+  <si>
+    <t>Mega Kangaskhan ex</t>
+  </si>
+  <si>
+    <t>Bouffalant</t>
+  </si>
+  <si>
+    <t>Tox Box</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>Mega Starmie</t>
+  </si>
+  <si>
+    <t>Team Rocket's Mewtwo ex</t>
+  </si>
+  <si>
+    <t>Okidogi</t>
+  </si>
+  <si>
+    <t>Bloodmoon Ursaluna</t>
+  </si>
+  <si>
+    <t>Doublade</t>
+  </si>
+  <si>
+    <t>Joltik Box</t>
+  </si>
+  <si>
+    <t>Joltik</t>
+  </si>
+  <si>
+    <t>Mega Zygarde</t>
+  </si>
+  <si>
+    <t>Mega Zygarde ex</t>
+  </si>
+  <si>
+    <t>Mega Sharpedo</t>
+  </si>
+  <si>
+    <t>Mega Sharpedo ex</t>
+  </si>
+  <si>
+    <t>Mega Abomasnow</t>
+  </si>
+  <si>
+    <t>Mega Abomasnow ex</t>
+  </si>
+  <si>
+    <t>Iono's Bellibolt</t>
+  </si>
+  <si>
+    <t>Iono's Bellibolt ex</t>
+  </si>
+  <si>
+    <t>Mega Dragonite</t>
+  </si>
+  <si>
+    <t>Mega Dragonite ex</t>
+  </si>
+  <si>
+    <t>Blissey</t>
+  </si>
+  <si>
+    <t>Blissey ex</t>
+  </si>
+  <si>
+    <t>Rocket Box</t>
+  </si>
+  <si>
+    <t>Mewtwo</t>
+  </si>
+  <si>
+    <t>Spidops</t>
+  </si>
+  <si>
+    <t>Team Rocket's Spidops</t>
+  </si>
+  <si>
+    <t>Mega Manectric ex</t>
+  </si>
+  <si>
+    <t>Mega Manectric</t>
+  </si>
+  <si>
+    <t>Azumarill</t>
+  </si>
+  <si>
+    <t>Azumarill ex</t>
+  </si>
+  <si>
+    <t>Decidueye</t>
+  </si>
+  <si>
+    <t>Decidueye ex</t>
+  </si>
+  <si>
+    <t>Bronzong</t>
+  </si>
+  <si>
+    <t>Mega Venusaur</t>
+  </si>
+  <si>
+    <t>Mega Venusaur ex</t>
+  </si>
+  <si>
+    <t>Yanmega</t>
+  </si>
+  <si>
+    <t>Yanmega ex</t>
+  </si>
+  <si>
+    <t>Eevee Box</t>
+  </si>
+  <si>
+    <t>Flareon ex</t>
+  </si>
+  <si>
+    <t>Feraligatr</t>
   </si>
 </sst>
 </file>
@@ -1225,4 +1574,1662 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}">
+  <dimension ref="A1:F82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" t="s">
+        <v>95</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D14" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D15" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" t="s">
+        <v>162</v>
+      </c>
+      <c r="D16" t="s">
+        <v>110</v>
+      </c>
+      <c r="E16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" t="s">
+        <v>162</v>
+      </c>
+      <c r="D17" t="s">
+        <v>111</v>
+      </c>
+      <c r="E17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" t="s">
+        <v>162</v>
+      </c>
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+      <c r="E19" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" t="s">
+        <v>162</v>
+      </c>
+      <c r="D20" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" t="s">
+        <v>95</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
+        <v>182</v>
+      </c>
+      <c r="C22" t="s">
+        <v>183</v>
+      </c>
+      <c r="D22" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" t="s">
+        <v>184</v>
+      </c>
+      <c r="D23" t="s">
+        <v>185</v>
+      </c>
+      <c r="E23" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>10</v>
+      </c>
+      <c r="B24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" t="s">
+        <v>95</v>
+      </c>
+      <c r="F24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>10</v>
+      </c>
+      <c r="B25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D25" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>10</v>
+      </c>
+      <c r="B26" t="s">
+        <v>123</v>
+      </c>
+      <c r="C26" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" t="s">
+        <v>95</v>
+      </c>
+      <c r="F26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>10</v>
+      </c>
+      <c r="B27" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" t="s">
+        <v>162</v>
+      </c>
+      <c r="D27" t="s">
+        <v>125</v>
+      </c>
+      <c r="E27" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" t="s">
+        <v>162</v>
+      </c>
+      <c r="D28" t="s">
+        <v>126</v>
+      </c>
+      <c r="E28" t="s">
+        <v>95</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" t="s">
+        <v>162</v>
+      </c>
+      <c r="D29" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" t="s">
+        <v>95</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" t="s">
+        <v>97</v>
+      </c>
+      <c r="E30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" t="s">
+        <v>162</v>
+      </c>
+      <c r="D31" t="s">
+        <v>129</v>
+      </c>
+      <c r="E31" t="s">
+        <v>95</v>
+      </c>
+      <c r="F31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" t="s">
+        <v>131</v>
+      </c>
+      <c r="E32" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>163</v>
+      </c>
+      <c r="C33" t="s">
+        <v>132</v>
+      </c>
+      <c r="D33" t="s">
+        <v>133</v>
+      </c>
+      <c r="E33" t="s">
+        <v>95</v>
+      </c>
+      <c r="F33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
+        <v>163</v>
+      </c>
+      <c r="C34" t="s">
+        <v>132</v>
+      </c>
+      <c r="D34" t="s">
+        <v>134</v>
+      </c>
+      <c r="E34" t="s">
+        <v>95</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>20</v>
+      </c>
+      <c r="B35" t="s">
+        <v>163</v>
+      </c>
+      <c r="C35" t="s">
+        <v>90</v>
+      </c>
+      <c r="D35" t="s">
+        <v>133</v>
+      </c>
+      <c r="E35" t="s">
+        <v>95</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>20</v>
+      </c>
+      <c r="B36" t="s">
+        <v>163</v>
+      </c>
+      <c r="C36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E36" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>30</v>
+      </c>
+      <c r="B37" t="s">
+        <v>163</v>
+      </c>
+      <c r="C37" t="s">
+        <v>162</v>
+      </c>
+      <c r="D37" t="s">
+        <v>133</v>
+      </c>
+      <c r="E37" t="s">
+        <v>95</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
+        <v>135</v>
+      </c>
+      <c r="C38" t="s">
+        <v>162</v>
+      </c>
+      <c r="D38" t="s">
+        <v>136</v>
+      </c>
+      <c r="E38" t="s">
+        <v>95</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>135</v>
+      </c>
+      <c r="C39" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>10</v>
+      </c>
+      <c r="B40" t="s">
+        <v>137</v>
+      </c>
+      <c r="C40" t="s">
+        <v>138</v>
+      </c>
+      <c r="D40" t="s">
+        <v>109</v>
+      </c>
+      <c r="E40" t="s">
+        <v>95</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>137</v>
+      </c>
+      <c r="C41" t="s">
+        <v>138</v>
+      </c>
+      <c r="D41" t="s">
+        <v>139</v>
+      </c>
+      <c r="E41" t="s">
+        <v>95</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>10</v>
+      </c>
+      <c r="B42" t="s">
+        <v>137</v>
+      </c>
+      <c r="C42" t="s">
+        <v>138</v>
+      </c>
+      <c r="D42" t="s">
+        <v>140</v>
+      </c>
+      <c r="E42" t="s">
+        <v>95</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>20</v>
+      </c>
+      <c r="B43" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" t="s">
+        <v>162</v>
+      </c>
+      <c r="D43" t="s">
+        <v>109</v>
+      </c>
+      <c r="E43" t="s">
+        <v>95</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>20</v>
+      </c>
+      <c r="B44" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" t="s">
+        <v>162</v>
+      </c>
+      <c r="D44" t="s">
+        <v>139</v>
+      </c>
+      <c r="E44" t="s">
+        <v>95</v>
+      </c>
+      <c r="F44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>141</v>
+      </c>
+      <c r="C45" t="s">
+        <v>162</v>
+      </c>
+      <c r="D45" t="s">
+        <v>141</v>
+      </c>
+      <c r="E45" t="s">
+        <v>95</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>10</v>
+      </c>
+      <c r="B46" t="s">
+        <v>142</v>
+      </c>
+      <c r="C46" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" t="s">
+        <v>95</v>
+      </c>
+      <c r="F46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>10</v>
+      </c>
+      <c r="B47" t="s">
+        <v>142</v>
+      </c>
+      <c r="C47" t="s">
+        <v>143</v>
+      </c>
+      <c r="D47" t="s">
+        <v>100</v>
+      </c>
+      <c r="E47" t="s">
+        <v>95</v>
+      </c>
+      <c r="F47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>20</v>
+      </c>
+      <c r="B48" t="s">
+        <v>142</v>
+      </c>
+      <c r="C48" t="s">
+        <v>97</v>
+      </c>
+      <c r="D48" t="s">
+        <v>144</v>
+      </c>
+      <c r="E48" t="s">
+        <v>95</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>20</v>
+      </c>
+      <c r="B49" t="s">
+        <v>142</v>
+      </c>
+      <c r="C49" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" t="s">
+        <v>97</v>
+      </c>
+      <c r="E49" t="s">
+        <v>95</v>
+      </c>
+      <c r="F49">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>30</v>
+      </c>
+      <c r="B50" t="s">
+        <v>142</v>
+      </c>
+      <c r="C50" t="s">
+        <v>162</v>
+      </c>
+      <c r="D50" t="s">
+        <v>144</v>
+      </c>
+      <c r="E50" t="s">
+        <v>95</v>
+      </c>
+      <c r="F50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>10</v>
+      </c>
+      <c r="B51" t="s">
+        <v>145</v>
+      </c>
+      <c r="C51" t="s">
+        <v>162</v>
+      </c>
+      <c r="D51" t="s">
+        <v>146</v>
+      </c>
+      <c r="E51" t="s">
+        <v>95</v>
+      </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>10</v>
+      </c>
+      <c r="B52" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" t="s">
+        <v>162</v>
+      </c>
+      <c r="D52" t="s">
+        <v>147</v>
+      </c>
+      <c r="E52" t="s">
+        <v>95</v>
+      </c>
+      <c r="F52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>149</v>
+      </c>
+      <c r="C53" t="s">
+        <v>90</v>
+      </c>
+      <c r="D53" t="s">
+        <v>150</v>
+      </c>
+      <c r="E53" t="s">
+        <v>95</v>
+      </c>
+      <c r="F53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>10</v>
+      </c>
+      <c r="B54" t="s">
+        <v>149</v>
+      </c>
+      <c r="C54" t="s">
+        <v>90</v>
+      </c>
+      <c r="D54" t="s">
+        <v>90</v>
+      </c>
+      <c r="E54" t="s">
+        <v>95</v>
+      </c>
+      <c r="F54">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>20</v>
+      </c>
+      <c r="B55" t="s">
+        <v>149</v>
+      </c>
+      <c r="C55" t="s">
+        <v>162</v>
+      </c>
+      <c r="D55" t="s">
+        <v>150</v>
+      </c>
+      <c r="E55" t="s">
+        <v>95</v>
+      </c>
+      <c r="F55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>10</v>
+      </c>
+      <c r="B56" t="s">
+        <v>151</v>
+      </c>
+      <c r="C56" t="s">
+        <v>162</v>
+      </c>
+      <c r="D56" t="s">
+        <v>110</v>
+      </c>
+      <c r="E56" t="s">
+        <v>95</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>10</v>
+      </c>
+      <c r="B57" t="s">
+        <v>151</v>
+      </c>
+      <c r="C57" t="s">
+        <v>162</v>
+      </c>
+      <c r="D57" t="s">
+        <v>152</v>
+      </c>
+      <c r="E57" t="s">
+        <v>95</v>
+      </c>
+      <c r="F57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>10</v>
+      </c>
+      <c r="B58" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" t="s">
+        <v>162</v>
+      </c>
+      <c r="D58" t="s">
+        <v>154</v>
+      </c>
+      <c r="E58" t="s">
+        <v>95</v>
+      </c>
+      <c r="F58">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>10</v>
+      </c>
+      <c r="B59" t="s">
+        <v>155</v>
+      </c>
+      <c r="C59" t="s">
+        <v>162</v>
+      </c>
+      <c r="D59" t="s">
+        <v>156</v>
+      </c>
+      <c r="E59" t="s">
+        <v>95</v>
+      </c>
+      <c r="F59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>10</v>
+      </c>
+      <c r="B60" t="s">
+        <v>155</v>
+      </c>
+      <c r="C60" t="s">
+        <v>162</v>
+      </c>
+      <c r="D60" t="s">
+        <v>159</v>
+      </c>
+      <c r="E60" t="s">
+        <v>95</v>
+      </c>
+      <c r="F60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
+        <v>158</v>
+      </c>
+      <c r="C61" t="s">
+        <v>162</v>
+      </c>
+      <c r="D61" t="s">
+        <v>159</v>
+      </c>
+      <c r="E61" t="s">
+        <v>95</v>
+      </c>
+      <c r="F61">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>10</v>
+      </c>
+      <c r="B62" t="s">
+        <v>158</v>
+      </c>
+      <c r="C62" t="s">
+        <v>162</v>
+      </c>
+      <c r="D62" t="s">
+        <v>160</v>
+      </c>
+      <c r="E62" t="s">
+        <v>95</v>
+      </c>
+      <c r="F62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>10</v>
+      </c>
+      <c r="B63" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63" t="s">
+        <v>162</v>
+      </c>
+      <c r="D63" t="s">
+        <v>157</v>
+      </c>
+      <c r="E63" t="s">
+        <v>95</v>
+      </c>
+      <c r="F63">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>10</v>
+      </c>
+      <c r="B64" t="s">
+        <v>165</v>
+      </c>
+      <c r="C64" t="s">
+        <v>162</v>
+      </c>
+      <c r="D64" t="s">
+        <v>165</v>
+      </c>
+      <c r="E64" t="s">
+        <v>95</v>
+      </c>
+      <c r="F64">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>10</v>
+      </c>
+      <c r="B65" t="s">
+        <v>166</v>
+      </c>
+      <c r="C65" t="s">
+        <v>162</v>
+      </c>
+      <c r="D65" t="s">
+        <v>166</v>
+      </c>
+      <c r="E65" t="s">
+        <v>95</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>10</v>
+      </c>
+      <c r="B66" t="s">
+        <v>187</v>
+      </c>
+      <c r="C66" t="s">
+        <v>162</v>
+      </c>
+      <c r="D66" t="s">
+        <v>186</v>
+      </c>
+      <c r="E66" t="s">
+        <v>95</v>
+      </c>
+      <c r="F66">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>10</v>
+      </c>
+      <c r="B67" t="s">
+        <v>167</v>
+      </c>
+      <c r="C67" t="s">
+        <v>162</v>
+      </c>
+      <c r="D67" t="s">
+        <v>167</v>
+      </c>
+      <c r="E67" t="s">
+        <v>95</v>
+      </c>
+      <c r="F67">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>10</v>
+      </c>
+      <c r="B68" t="s">
+        <v>168</v>
+      </c>
+      <c r="C68" t="s">
+        <v>162</v>
+      </c>
+      <c r="D68" t="s">
+        <v>169</v>
+      </c>
+      <c r="E68" t="s">
+        <v>95</v>
+      </c>
+      <c r="F68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>10</v>
+      </c>
+      <c r="B69" t="s">
+        <v>170</v>
+      </c>
+      <c r="C69" t="s">
+        <v>162</v>
+      </c>
+      <c r="D69" t="s">
+        <v>171</v>
+      </c>
+      <c r="E69" t="s">
+        <v>95</v>
+      </c>
+      <c r="F69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>10</v>
+      </c>
+      <c r="B70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C70" t="s">
+        <v>162</v>
+      </c>
+      <c r="D70" t="s">
+        <v>173</v>
+      </c>
+      <c r="E70" t="s">
+        <v>95</v>
+      </c>
+      <c r="F70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>10</v>
+      </c>
+      <c r="B71" t="s">
+        <v>174</v>
+      </c>
+      <c r="C71" t="s">
+        <v>162</v>
+      </c>
+      <c r="D71" t="s">
+        <v>175</v>
+      </c>
+      <c r="E71" t="s">
+        <v>95</v>
+      </c>
+      <c r="F71">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>10</v>
+      </c>
+      <c r="B72" t="s">
+        <v>176</v>
+      </c>
+      <c r="C72" t="s">
+        <v>162</v>
+      </c>
+      <c r="D72" t="s">
+        <v>177</v>
+      </c>
+      <c r="E72" t="s">
+        <v>95</v>
+      </c>
+      <c r="F72">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>10</v>
+      </c>
+      <c r="B73" t="s">
+        <v>178</v>
+      </c>
+      <c r="C73" t="s">
+        <v>162</v>
+      </c>
+      <c r="D73" t="s">
+        <v>179</v>
+      </c>
+      <c r="E73" t="s">
+        <v>95</v>
+      </c>
+      <c r="F73">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>10</v>
+      </c>
+      <c r="B74" t="s">
+        <v>180</v>
+      </c>
+      <c r="C74" t="s">
+        <v>162</v>
+      </c>
+      <c r="D74" t="s">
+        <v>181</v>
+      </c>
+      <c r="E74" t="s">
+        <v>95</v>
+      </c>
+      <c r="F74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>10</v>
+      </c>
+      <c r="B75" t="s">
+        <v>188</v>
+      </c>
+      <c r="C75" t="s">
+        <v>162</v>
+      </c>
+      <c r="D75" t="s">
+        <v>189</v>
+      </c>
+      <c r="E75" t="s">
+        <v>95</v>
+      </c>
+      <c r="F75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>10</v>
+      </c>
+      <c r="B76" t="s">
+        <v>190</v>
+      </c>
+      <c r="C76" t="s">
+        <v>162</v>
+      </c>
+      <c r="D76" t="s">
+        <v>191</v>
+      </c>
+      <c r="E76" t="s">
+        <v>95</v>
+      </c>
+      <c r="F76">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>10</v>
+      </c>
+      <c r="B77" t="s">
+        <v>192</v>
+      </c>
+      <c r="C77" t="s">
+        <v>162</v>
+      </c>
+      <c r="D77" t="s">
+        <v>192</v>
+      </c>
+      <c r="E77" t="s">
+        <v>95</v>
+      </c>
+      <c r="F77">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>10</v>
+      </c>
+      <c r="B78" t="s">
+        <v>193</v>
+      </c>
+      <c r="C78" t="s">
+        <v>162</v>
+      </c>
+      <c r="D78" t="s">
+        <v>194</v>
+      </c>
+      <c r="E78" t="s">
+        <v>95</v>
+      </c>
+      <c r="F78">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>10</v>
+      </c>
+      <c r="B79" t="s">
+        <v>195</v>
+      </c>
+      <c r="C79" t="s">
+        <v>162</v>
+      </c>
+      <c r="D79" t="s">
+        <v>196</v>
+      </c>
+      <c r="E79" t="s">
+        <v>95</v>
+      </c>
+      <c r="F79">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>10</v>
+      </c>
+      <c r="B80" t="s">
+        <v>197</v>
+      </c>
+      <c r="C80" t="s">
+        <v>162</v>
+      </c>
+      <c r="D80" t="s">
+        <v>198</v>
+      </c>
+      <c r="E80" t="s">
+        <v>95</v>
+      </c>
+      <c r="F80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>10</v>
+      </c>
+      <c r="B81" t="s">
+        <v>197</v>
+      </c>
+      <c r="C81" t="s">
+        <v>162</v>
+      </c>
+      <c r="D81" t="s">
+        <v>152</v>
+      </c>
+      <c r="E81" t="s">
+        <v>95</v>
+      </c>
+      <c r="F81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>10</v>
+      </c>
+      <c r="B82" t="s">
+        <v>199</v>
+      </c>
+      <c r="C82" t="s">
+        <v>162</v>
+      </c>
+      <c r="D82" t="s">
+        <v>199</v>
+      </c>
+      <c r="E82" t="s">
+        <v>95</v>
+      </c>
+      <c r="F82">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F63" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add classification sync and tournament analytics foundation
</commit_message>
<xml_diff>
--- a/metadata/metadata.xlsx
+++ b/metadata/metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madis\Documents\pokemon_scraper\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBBD407-B975-4D99-BB92-DD1840BF4EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86E36E6-4B6F-455B-B29A-A1B31248EE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="archetypes" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">archetypes!$A$1:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">archetypes!$A$1:$F$76</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="210">
   <si>
     <t>tournament_id</t>
   </si>
@@ -611,12 +611,6 @@
     <t>Bronzong</t>
   </si>
   <si>
-    <t>Mega Venusaur</t>
-  </si>
-  <si>
-    <t>Mega Venusaur ex</t>
-  </si>
-  <si>
     <t>Yanmega</t>
   </si>
   <si>
@@ -630,6 +624,42 @@
   </si>
   <si>
     <t>Feraligatr</t>
+  </si>
+  <si>
+    <t>Venusaur</t>
+  </si>
+  <si>
+    <t>Venusaur ex</t>
+  </si>
+  <si>
+    <t>Metang</t>
+  </si>
+  <si>
+    <t>Basic Box</t>
+  </si>
+  <si>
+    <t>Meowth ex</t>
+  </si>
+  <si>
+    <t>&lt;</t>
+  </si>
+  <si>
+    <t>Palafin</t>
+  </si>
+  <si>
+    <t>Palafin ex</t>
+  </si>
+  <si>
+    <t>Cinccino</t>
+  </si>
+  <si>
+    <t>Cinccino ex</t>
+  </si>
+  <si>
+    <t>Hydreigon</t>
+  </si>
+  <si>
+    <t>Hydreigon ex</t>
   </si>
 </sst>
 </file>
@@ -1578,7 +1608,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -1813,19 +1843,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
         <v>162</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E12" t="s">
         <v>95</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1833,19 +1863,19 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>201</v>
       </c>
       <c r="C13" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="D13" t="s">
-        <v>104</v>
+        <v>159</v>
       </c>
       <c r="E13" t="s">
         <v>95</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1853,13 +1883,13 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
+        <v>201</v>
+      </c>
+      <c r="C14" t="s">
         <v>105</v>
       </c>
-      <c r="C14" t="s">
-        <v>162</v>
-      </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>202</v>
       </c>
       <c r="E14" t="s">
         <v>95</v>
@@ -1873,53 +1903,53 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>201</v>
       </c>
       <c r="C15" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E15" t="s">
         <v>95</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>201</v>
       </c>
       <c r="C16" t="s">
         <v>162</v>
       </c>
       <c r="D16" t="s">
-        <v>110</v>
+        <v>159</v>
       </c>
       <c r="E16" t="s">
         <v>95</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>106</v>
+        <v>201</v>
       </c>
       <c r="C17" t="s">
         <v>162</v>
       </c>
       <c r="D17" t="s">
-        <v>111</v>
+        <v>202</v>
       </c>
       <c r="E17" t="s">
         <v>95</v>
@@ -1930,10 +1960,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>201</v>
       </c>
       <c r="C18" t="s">
         <v>162</v>
@@ -1942,7 +1972,7 @@
         <v>113</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>203</v>
       </c>
       <c r="F18">
         <v>3</v>
@@ -1950,22 +1980,22 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>201</v>
       </c>
       <c r="C19" t="s">
         <v>162</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E19" t="s">
         <v>95</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1973,19 +2003,19 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
         <v>162</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E20" t="s">
         <v>95</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1993,19 +2023,19 @@
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
         <v>162</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
         <v>95</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2013,13 +2043,13 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>182</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
       <c r="D22" t="s">
-        <v>164</v>
+        <v>111</v>
       </c>
       <c r="E22" t="s">
         <v>95</v>
@@ -2033,13 +2063,13 @@
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>182</v>
+        <v>112</v>
       </c>
       <c r="C23" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="D23" t="s">
-        <v>185</v>
+        <v>113</v>
       </c>
       <c r="E23" t="s">
         <v>95</v>
@@ -2053,13 +2083,13 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C24" t="s">
         <v>162</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E24" t="s">
         <v>95</v>
@@ -2073,13 +2103,13 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C25" t="s">
         <v>162</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E25" t="s">
         <v>95</v>
@@ -2093,19 +2123,19 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C26" t="s">
         <v>162</v>
       </c>
       <c r="D26" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E26" t="s">
         <v>95</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2113,19 +2143,19 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>182</v>
       </c>
       <c r="C27" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="D27" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="E27" t="s">
         <v>95</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2133,19 +2163,19 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>182</v>
       </c>
       <c r="C28" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>185</v>
       </c>
       <c r="E28" t="s">
         <v>95</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2153,19 +2183,19 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C29" t="s">
         <v>162</v>
       </c>
       <c r="D29" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="E29" t="s">
         <v>95</v>
       </c>
       <c r="F29">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2173,19 +2203,19 @@
         <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C30" t="s">
         <v>162</v>
       </c>
       <c r="D30" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="E30" t="s">
         <v>95</v>
       </c>
       <c r="F30">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2193,19 +2223,19 @@
         <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C31" t="s">
         <v>162</v>
       </c>
       <c r="D31" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E31" t="s">
         <v>95</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2213,19 +2243,19 @@
         <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
         <v>162</v>
       </c>
       <c r="D32" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E32" t="s">
         <v>95</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2233,19 +2263,19 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="C33" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="D33" t="s">
-        <v>133</v>
+        <v>200</v>
       </c>
       <c r="E33" t="s">
         <v>95</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2253,33 +2283,33 @@
         <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>163</v>
+        <v>126</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>162</v>
       </c>
       <c r="D34" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="E34" t="s">
         <v>95</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="C35" t="s">
         <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E35" t="s">
         <v>95</v>
@@ -2290,10 +2320,10 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="C36" t="s">
         <v>90</v>
@@ -2310,16 +2340,16 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s">
         <v>162</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E37" t="s">
         <v>95</v>
@@ -2330,16 +2360,16 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C38" t="s">
         <v>162</v>
       </c>
       <c r="D38" t="s">
-        <v>136</v>
+        <v>97</v>
       </c>
       <c r="E38" t="s">
         <v>95</v>
@@ -2350,22 +2380,22 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C39" t="s">
         <v>162</v>
       </c>
       <c r="D39" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="E39" t="s">
         <v>95</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2373,19 +2403,19 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C40" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="D40" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="E40" t="s">
         <v>95</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2393,13 +2423,13 @@
         <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D41" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E41" t="s">
         <v>95</v>
@@ -2413,19 +2443,19 @@
         <v>10</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="C42" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D42" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E42" t="s">
         <v>95</v>
       </c>
       <c r="F42">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2433,19 +2463,19 @@
         <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="C43" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D43" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="E43" t="s">
         <v>95</v>
       </c>
       <c r="F43">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2453,33 +2483,33 @@
         <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>163</v>
       </c>
       <c r="C44" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="E44" t="s">
         <v>95</v>
       </c>
       <c r="F44">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="C45" t="s">
         <v>162</v>
       </c>
       <c r="D45" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="E45" t="s">
         <v>95</v>
@@ -2493,13 +2523,13 @@
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C46" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="E46" t="s">
         <v>95</v>
@@ -2513,13 +2543,13 @@
         <v>10</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="E47" t="s">
         <v>95</v>
@@ -2530,16 +2560,16 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="D48" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E48" t="s">
         <v>95</v>
@@ -2550,16 +2580,16 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C49" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="D49" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="E49" t="s">
         <v>95</v>
@@ -2570,16 +2600,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B50" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C50" t="s">
-        <v>162</v>
+        <v>103</v>
       </c>
       <c r="D50" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="E50" t="s">
         <v>95</v>
@@ -2590,16 +2620,16 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C51" t="s">
-        <v>162</v>
+        <v>103</v>
       </c>
       <c r="D51" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E51" t="s">
         <v>95</v>
@@ -2610,16 +2640,16 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B52" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="C52" t="s">
-        <v>162</v>
+        <v>103</v>
       </c>
       <c r="D52" t="s">
-        <v>147</v>
+        <v>107</v>
       </c>
       <c r="E52" t="s">
         <v>95</v>
@@ -2630,16 +2660,16 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B53" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C53" t="s">
-        <v>90</v>
+        <v>198</v>
       </c>
       <c r="D53" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="E53" t="s">
         <v>95</v>
@@ -2650,16 +2680,16 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B54" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>198</v>
       </c>
       <c r="D54" t="s">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="E54" t="s">
         <v>95</v>
@@ -2670,16 +2700,16 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B55" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C55" t="s">
-        <v>162</v>
+        <v>198</v>
       </c>
       <c r="D55" t="s">
-        <v>150</v>
+        <v>199</v>
       </c>
       <c r="E55" t="s">
         <v>95</v>
@@ -2690,36 +2720,36 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B56" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C56" t="s">
         <v>162</v>
       </c>
       <c r="D56" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E56" t="s">
         <v>95</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B57" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C57" t="s">
         <v>162</v>
       </c>
       <c r="D57" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="E57" t="s">
         <v>95</v>
@@ -2733,13 +2763,13 @@
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C58" t="s">
         <v>162</v>
       </c>
       <c r="D58" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E58" t="s">
         <v>95</v>
@@ -2753,13 +2783,13 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="C59" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="D59" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="E59" t="s">
         <v>95</v>
@@ -2773,13 +2803,13 @@
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="C60" t="s">
-        <v>162</v>
+        <v>143</v>
       </c>
       <c r="D60" t="s">
-        <v>159</v>
+        <v>100</v>
       </c>
       <c r="E60" t="s">
         <v>95</v>
@@ -2790,16 +2820,16 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C61" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="D61" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="E61" t="s">
         <v>95</v>
@@ -2810,16 +2840,16 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C62" t="s">
-        <v>162</v>
+        <v>97</v>
       </c>
       <c r="D62" t="s">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="E62" t="s">
         <v>95</v>
@@ -2830,22 +2860,22 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B63" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="C63" t="s">
         <v>162</v>
       </c>
       <c r="D63" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="E63" t="s">
         <v>95</v>
       </c>
       <c r="F63">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2853,19 +2883,19 @@
         <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C64" t="s">
         <v>162</v>
       </c>
       <c r="D64" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="E64" t="s">
         <v>95</v>
       </c>
       <c r="F64">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2873,13 +2903,13 @@
         <v>10</v>
       </c>
       <c r="B65" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="C65" t="s">
         <v>162</v>
       </c>
       <c r="D65" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="E65" t="s">
         <v>95</v>
@@ -2893,13 +2923,13 @@
         <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>187</v>
+        <v>149</v>
       </c>
       <c r="C66" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="E66" t="s">
         <v>95</v>
@@ -2913,33 +2943,33 @@
         <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
       <c r="C67" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>167</v>
+        <v>90</v>
       </c>
       <c r="E67" t="s">
         <v>95</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B68" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="C68" t="s">
         <v>162</v>
       </c>
       <c r="D68" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="E68" t="s">
         <v>95</v>
@@ -2953,19 +2983,19 @@
         <v>10</v>
       </c>
       <c r="B69" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C69" t="s">
         <v>162</v>
       </c>
       <c r="D69" t="s">
-        <v>171</v>
+        <v>110</v>
       </c>
       <c r="E69" t="s">
         <v>95</v>
       </c>
       <c r="F69">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2973,13 +3003,13 @@
         <v>10</v>
       </c>
       <c r="B70" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="C70" t="s">
         <v>162</v>
       </c>
       <c r="D70" t="s">
-        <v>173</v>
+        <v>152</v>
       </c>
       <c r="E70" t="s">
         <v>95</v>
@@ -2993,13 +3023,13 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="C71" t="s">
         <v>162</v>
       </c>
       <c r="D71" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="E71" t="s">
         <v>95</v>
@@ -3013,13 +3043,13 @@
         <v>10</v>
       </c>
       <c r="B72" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="C72" t="s">
         <v>162</v>
       </c>
       <c r="D72" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="E72" t="s">
         <v>95</v>
@@ -3033,13 +3063,13 @@
         <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="C73" t="s">
         <v>162</v>
       </c>
       <c r="D73" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="E73" t="s">
         <v>95</v>
@@ -3053,13 +3083,13 @@
         <v>10</v>
       </c>
       <c r="B74" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="C74" t="s">
         <v>162</v>
       </c>
       <c r="D74" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="E74" t="s">
         <v>95</v>
@@ -3073,13 +3103,13 @@
         <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="C75" t="s">
         <v>162</v>
       </c>
       <c r="D75" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="E75" t="s">
         <v>95</v>
@@ -3093,19 +3123,19 @@
         <v>10</v>
       </c>
       <c r="B76" t="s">
-        <v>190</v>
+        <v>161</v>
       </c>
       <c r="C76" t="s">
         <v>162</v>
       </c>
       <c r="D76" t="s">
-        <v>191</v>
+        <v>157</v>
       </c>
       <c r="E76" t="s">
         <v>95</v>
       </c>
       <c r="F76">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3113,19 +3143,19 @@
         <v>10</v>
       </c>
       <c r="B77" t="s">
-        <v>192</v>
+        <v>165</v>
       </c>
       <c r="C77" t="s">
         <v>162</v>
       </c>
       <c r="D77" t="s">
-        <v>192</v>
+        <v>165</v>
       </c>
       <c r="E77" t="s">
         <v>95</v>
       </c>
       <c r="F77">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -3133,13 +3163,13 @@
         <v>10</v>
       </c>
       <c r="B78" t="s">
-        <v>193</v>
+        <v>166</v>
       </c>
       <c r="C78" t="s">
         <v>162</v>
       </c>
       <c r="D78" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="E78" t="s">
         <v>95</v>
@@ -3153,13 +3183,13 @@
         <v>10</v>
       </c>
       <c r="B79" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C79" t="s">
         <v>162</v>
       </c>
       <c r="D79" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="E79" t="s">
         <v>95</v>
@@ -3173,19 +3203,19 @@
         <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>197</v>
+        <v>167</v>
       </c>
       <c r="C80" t="s">
         <v>162</v>
       </c>
       <c r="D80" t="s">
-        <v>198</v>
+        <v>167</v>
       </c>
       <c r="E80" t="s">
         <v>95</v>
       </c>
       <c r="F80">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -3193,13 +3223,13 @@
         <v>10</v>
       </c>
       <c r="B81" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C81" t="s">
         <v>162</v>
       </c>
       <c r="D81" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="E81" t="s">
         <v>95</v>
@@ -3213,13 +3243,13 @@
         <v>10</v>
       </c>
       <c r="B82" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="C82" t="s">
         <v>162</v>
       </c>
       <c r="D82" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
       <c r="E82" t="s">
         <v>95</v>
@@ -3228,8 +3258,528 @@
         <v>2</v>
       </c>
     </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>172</v>
+      </c>
+      <c r="C83" t="s">
+        <v>162</v>
+      </c>
+      <c r="D83" t="s">
+        <v>173</v>
+      </c>
+      <c r="E83" t="s">
+        <v>95</v>
+      </c>
+      <c r="F83">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>10</v>
+      </c>
+      <c r="B84" t="s">
+        <v>174</v>
+      </c>
+      <c r="C84" t="s">
+        <v>162</v>
+      </c>
+      <c r="D84" t="s">
+        <v>175</v>
+      </c>
+      <c r="E84" t="s">
+        <v>95</v>
+      </c>
+      <c r="F84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>10</v>
+      </c>
+      <c r="B85" t="s">
+        <v>176</v>
+      </c>
+      <c r="C85" t="s">
+        <v>162</v>
+      </c>
+      <c r="D85" t="s">
+        <v>177</v>
+      </c>
+      <c r="E85" t="s">
+        <v>95</v>
+      </c>
+      <c r="F85">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>10</v>
+      </c>
+      <c r="B86" t="s">
+        <v>178</v>
+      </c>
+      <c r="C86" t="s">
+        <v>162</v>
+      </c>
+      <c r="D86" t="s">
+        <v>179</v>
+      </c>
+      <c r="E86" t="s">
+        <v>95</v>
+      </c>
+      <c r="F86">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>10</v>
+      </c>
+      <c r="B87" t="s">
+        <v>180</v>
+      </c>
+      <c r="C87" t="s">
+        <v>162</v>
+      </c>
+      <c r="D87" t="s">
+        <v>181</v>
+      </c>
+      <c r="E87" t="s">
+        <v>95</v>
+      </c>
+      <c r="F87">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>10</v>
+      </c>
+      <c r="B88" t="s">
+        <v>188</v>
+      </c>
+      <c r="C88" t="s">
+        <v>162</v>
+      </c>
+      <c r="D88" t="s">
+        <v>189</v>
+      </c>
+      <c r="E88" t="s">
+        <v>95</v>
+      </c>
+      <c r="F88">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>10</v>
+      </c>
+      <c r="B89" t="s">
+        <v>190</v>
+      </c>
+      <c r="C89" t="s">
+        <v>162</v>
+      </c>
+      <c r="D89" t="s">
+        <v>191</v>
+      </c>
+      <c r="E89" t="s">
+        <v>95</v>
+      </c>
+      <c r="F89">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>10</v>
+      </c>
+      <c r="B90" t="s">
+        <v>192</v>
+      </c>
+      <c r="C90" t="s">
+        <v>162</v>
+      </c>
+      <c r="D90" t="s">
+        <v>192</v>
+      </c>
+      <c r="E90" t="s">
+        <v>95</v>
+      </c>
+      <c r="F90">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>10</v>
+      </c>
+      <c r="B91" t="s">
+        <v>193</v>
+      </c>
+      <c r="C91" t="s">
+        <v>162</v>
+      </c>
+      <c r="D91" t="s">
+        <v>194</v>
+      </c>
+      <c r="E91" t="s">
+        <v>95</v>
+      </c>
+      <c r="F91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>10</v>
+      </c>
+      <c r="B92" t="s">
+        <v>195</v>
+      </c>
+      <c r="C92" t="s">
+        <v>162</v>
+      </c>
+      <c r="D92" t="s">
+        <v>196</v>
+      </c>
+      <c r="E92" t="s">
+        <v>95</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>10</v>
+      </c>
+      <c r="B93" t="s">
+        <v>195</v>
+      </c>
+      <c r="C93" t="s">
+        <v>162</v>
+      </c>
+      <c r="D93" t="s">
+        <v>152</v>
+      </c>
+      <c r="E93" t="s">
+        <v>95</v>
+      </c>
+      <c r="F93">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>10</v>
+      </c>
+      <c r="B94" t="s">
+        <v>197</v>
+      </c>
+      <c r="C94" t="s">
+        <v>162</v>
+      </c>
+      <c r="D94" t="s">
+        <v>197</v>
+      </c>
+      <c r="E94" t="s">
+        <v>95</v>
+      </c>
+      <c r="F94">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>10</v>
+      </c>
+      <c r="B95" t="s">
+        <v>105</v>
+      </c>
+      <c r="C95" t="s">
+        <v>152</v>
+      </c>
+      <c r="D95" t="s">
+        <v>108</v>
+      </c>
+      <c r="E95" t="s">
+        <v>95</v>
+      </c>
+      <c r="F95">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>10</v>
+      </c>
+      <c r="B96" t="s">
+        <v>105</v>
+      </c>
+      <c r="C96" t="s">
+        <v>152</v>
+      </c>
+      <c r="D96" t="s">
+        <v>152</v>
+      </c>
+      <c r="E96" t="s">
+        <v>95</v>
+      </c>
+      <c r="F96">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>20</v>
+      </c>
+      <c r="B97" t="s">
+        <v>105</v>
+      </c>
+      <c r="C97" t="s">
+        <v>162</v>
+      </c>
+      <c r="D97" t="s">
+        <v>108</v>
+      </c>
+      <c r="E97" t="s">
+        <v>95</v>
+      </c>
+      <c r="F97">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>20</v>
+      </c>
+      <c r="B98" t="s">
+        <v>105</v>
+      </c>
+      <c r="C98" t="s">
+        <v>162</v>
+      </c>
+      <c r="D98" t="s">
+        <v>109</v>
+      </c>
+      <c r="E98" t="s">
+        <v>95</v>
+      </c>
+      <c r="F98">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>10</v>
+      </c>
+      <c r="B99" t="s">
+        <v>204</v>
+      </c>
+      <c r="C99" t="s">
+        <v>162</v>
+      </c>
+      <c r="D99" t="s">
+        <v>205</v>
+      </c>
+      <c r="E99" t="s">
+        <v>95</v>
+      </c>
+      <c r="F99">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>10</v>
+      </c>
+      <c r="B100" t="s">
+        <v>206</v>
+      </c>
+      <c r="C100" t="s">
+        <v>162</v>
+      </c>
+      <c r="D100" t="s">
+        <v>207</v>
+      </c>
+      <c r="E100" t="s">
+        <v>95</v>
+      </c>
+      <c r="F100">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>10</v>
+      </c>
+      <c r="B101" t="s">
+        <v>96</v>
+      </c>
+      <c r="C101" t="s">
+        <v>143</v>
+      </c>
+      <c r="D101" t="s">
+        <v>89</v>
+      </c>
+      <c r="E101" t="s">
+        <v>95</v>
+      </c>
+      <c r="F101">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>10</v>
+      </c>
+      <c r="B102" t="s">
+        <v>96</v>
+      </c>
+      <c r="C102" t="s">
+        <v>143</v>
+      </c>
+      <c r="D102" t="s">
+        <v>100</v>
+      </c>
+      <c r="E102" t="s">
+        <v>95</v>
+      </c>
+      <c r="F102">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>20</v>
+      </c>
+      <c r="B103" t="s">
+        <v>96</v>
+      </c>
+      <c r="C103" t="s">
+        <v>162</v>
+      </c>
+      <c r="D103" t="s">
+        <v>89</v>
+      </c>
+      <c r="E103" t="s">
+        <v>95</v>
+      </c>
+      <c r="F103">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>10</v>
+      </c>
+      <c r="B104" t="s">
+        <v>208</v>
+      </c>
+      <c r="C104" t="s">
+        <v>162</v>
+      </c>
+      <c r="D104" t="s">
+        <v>209</v>
+      </c>
+      <c r="E104" t="s">
+        <v>95</v>
+      </c>
+      <c r="F104">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>10</v>
+      </c>
+      <c r="B105" t="s">
+        <v>138</v>
+      </c>
+      <c r="C105" t="s">
+        <v>132</v>
+      </c>
+      <c r="D105" t="s">
+        <v>140</v>
+      </c>
+      <c r="E105" t="s">
+        <v>95</v>
+      </c>
+      <c r="F105">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>10</v>
+      </c>
+      <c r="B106" t="s">
+        <v>138</v>
+      </c>
+      <c r="C106" t="s">
+        <v>132</v>
+      </c>
+      <c r="D106" t="s">
+        <v>132</v>
+      </c>
+      <c r="E106" t="s">
+        <v>95</v>
+      </c>
+      <c r="F106">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>20</v>
+      </c>
+      <c r="B107" t="s">
+        <v>138</v>
+      </c>
+      <c r="C107" t="s">
+        <v>90</v>
+      </c>
+      <c r="D107" t="s">
+        <v>140</v>
+      </c>
+      <c r="E107" t="s">
+        <v>95</v>
+      </c>
+      <c r="F107">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>20</v>
+      </c>
+      <c r="B108" t="s">
+        <v>138</v>
+      </c>
+      <c r="C108" t="s">
+        <v>90</v>
+      </c>
+      <c r="D108" t="s">
+        <v>90</v>
+      </c>
+      <c r="E108" t="s">
+        <v>95</v>
+      </c>
+      <c r="F108">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F63" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}"/>
+  <autoFilter ref="A1:F76" xr:uid="{6109B466-147E-4821-8C23-D053C5656631}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>